<commit_message>
Bland svarmulighederne, så facit ikke altid står først
Det rigtige svar stod som A i alle 30 spørgsmål, fordi det var sådan de blev
skrevet ned. byg_quiz.py blander nu de fire muligheder med en fast seed, så alle
formater får præcis samme rækkefølge, og scriptet afviser en skæv fordeling.
Facit ligger nu 6 gange på A, 7 på B, 10 på C og 7 på D.

Alle udgaver er bygget om: den interaktive side, regnearket, PowerPointen,
Word- og tekstudgaven, de 30 billeder og overbliks-PDF'en. Regnearkets
facitkolonne er sammenlignet med kilden bagefter, og siden er afprøvet i browser
igen — koderne afkoder stadig præcis rigtigt.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VgEVctXq3tNeZxt6iAFBPu
</commit_message>
<xml_diff>
--- a/facit/kahoot-statistik-2026-09-11.xlsx
+++ b/facit/kahoot-statistik-2026-09-11.xlsx
@@ -529,29 +529,29 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
           <t>6</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>5</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>8</t>
         </is>
       </c>
       <c r="G9" s="4" t="n">
         <v>20</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -565,29 +565,29 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
           <t>5</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>13</t>
         </is>
       </c>
       <c r="G10" s="4" t="n">
         <v>20</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -606,12 +606,12 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
           <t>13</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -637,29 +637,29 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
           <t>7</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>49</t>
-        </is>
-      </c>
       <c r="G12" s="4" t="n">
         <v>30</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -673,29 +673,29 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
       <c r="G13" s="4" t="n">
         <v>30</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
@@ -709,29 +709,29 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
           <t>9</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
       <c r="G14" s="4" t="n">
         <v>30</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
@@ -745,29 +745,29 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
+          <t>Gennemsnit, median, typetal, sum og antal</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
           <t>Mindste, nedre kvartil, median, øvre kvartil, største</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>Mindste, gennemsnit, median, typetal, største</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>De fem mindste tal i datasættet</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>Gennemsnit, median, typetal, sum og antal</t>
-        </is>
-      </c>
       <c r="G15" s="4" t="n">
         <v>30</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
@@ -781,14 +781,14 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
+          <t>25 %</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
           <t>50 %</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>25 %</t>
-        </is>
-      </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
           <t>75 %</t>
@@ -803,7 +803,7 @@
         <v>30</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
@@ -817,19 +817,19 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
           <t>6</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
           <t>7</t>
@@ -839,7 +839,7 @@
         <v>30</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18">
@@ -853,29 +853,29 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
+          <t>Den stiger lidt</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Den falder</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Den bliver dobbelt så stor</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
           <t>Ingenting</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>Den bliver dobbelt så stor</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>Den stiger lidt</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>Den falder</t>
-        </is>
-      </c>
       <c r="G18" s="4" t="n">
         <v>30</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19">
@@ -889,29 +889,29 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
           <t>8</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
       <c r="G19" s="4" t="n">
         <v>30</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
@@ -925,29 +925,29 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
+          <t>90°</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>15°</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
           <t>135°</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>150°</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>90°</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>15°</t>
-        </is>
-      </c>
       <c r="G20" s="4" t="n">
         <v>30</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
@@ -961,29 +961,29 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
+          <t>80°</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>45°</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>8°</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
           <t>72°</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>80°</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>8°</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>45°</t>
-        </is>
-      </c>
       <c r="G21" s="4" t="n">
         <v>30</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22">
@@ -997,19 +997,19 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
+          <t>40 %</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>10 %</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
           <t>25 %</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>10 %</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>40 %</t>
-        </is>
-      </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
           <t>15 %</t>
@@ -1019,7 +1019,7 @@
         <v>30</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23">
@@ -1033,29 +1033,29 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
+          <t>Svømning</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Andet</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
           <t>Håndbold</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="F23" s="4" t="inlineStr">
         <is>
           <t>Fodbold</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>Svømning</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>Andet</t>
         </is>
       </c>
       <c r="G23" s="4" t="n">
         <v>20</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24">
@@ -1069,29 +1069,29 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
+          <t>360 %</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Gennemsnittet</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
           <t>100 %</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>360 %</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="F24" s="4" t="inlineStr">
         <is>
           <t>Antallet af observationer</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>Gennemsnittet</t>
         </is>
       </c>
       <c r="G24" s="4" t="n">
         <v>20</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25">
@@ -1141,29 +1141,29 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
+          <t>Omkring 155 cm</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Omkring 160 cm</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
           <t>Omkring 172 cm</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>Omkring 160 cm</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>Omkring 180 cm</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t>Omkring 155 cm</t>
-        </is>
-      </c>
       <c r="G26" s="4" t="n">
         <v>30</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27">
@@ -1177,29 +1177,29 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
+          <t>25 %</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
           <t>80 %</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>25 %</t>
-        </is>
-      </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
+          <t>35 %</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
           <t>100 %</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>35 %</t>
-        </is>
-      </c>
       <c r="G27" s="4" t="n">
         <v>30</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28">
@@ -1213,17 +1213,17 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
+          <t>2-4 timer</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>0-2 timer</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
           <t>4-6 timer</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>0-2 timer</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>2-4 timer</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
@@ -1235,7 +1235,7 @@
         <v>20</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29">
@@ -1249,29 +1249,29 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
+          <t>4 gange</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
           <t>2 gange</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>3 gange</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
         <is>
           <t>1 gang</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>3 gange</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>4 gange</t>
         </is>
       </c>
       <c r="G29" s="4" t="n">
         <v>20</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30">
@@ -1285,19 +1285,19 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
+          <t>7 ud af 36</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>1 ud af 36</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
           <t>6 ud af 36</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>1 ud af 36</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>7 ud af 36</t>
-        </is>
-      </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
           <t>1 ud af 12</t>
@@ -1307,7 +1307,7 @@
         <v>30</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31">
@@ -1367,12 +1367,12 @@
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
+          <t>2 ud af 36</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
           <t>12 ud af 36</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>2 ud af 36</t>
         </is>
       </c>
       <c r="G32" s="4" t="n">
@@ -1393,29 +1393,29 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
+          <t>21 procentpoint</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
           <t>6 procentpoint</t>
         </is>
       </c>
-      <c r="D33" s="4" t="inlineStr">
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>6 procent</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
         <is>
           <t>40 procentpoint</t>
         </is>
       </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>6 procent</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>21 procentpoint</t>
-        </is>
-      </c>
       <c r="G33" s="4" t="n">
         <v>30</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34">
@@ -1434,17 +1434,17 @@
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
+          <t>36 %</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>21 %</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
           <t>6 %</t>
-        </is>
-      </c>
-      <c r="E34" s="4" t="inlineStr">
-        <is>
-          <t>21 %</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="inlineStr">
-        <is>
-          <t>36 %</t>
         </is>
       </c>
       <c r="G34" s="4" t="n">
@@ -1465,29 +1465,29 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
+          <t>38 %</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
           <t>9,5 %</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
-          <t>38 %</t>
-        </is>
-      </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
+          <t>90,5 %</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
           <t>10,5 %</t>
         </is>
       </c>
-      <c r="F35" s="4" t="inlineStr">
-        <is>
-          <t>90,5 %</t>
-        </is>
-      </c>
       <c r="G35" s="4" t="n">
         <v>30</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36">
@@ -1506,17 +1506,17 @@
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
+          <t>Ingenting — tallene er jo de samme</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>Diagrammet bliver ulovligt</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
           <t>Forskellene ser mindre ud, end de er</t>
-        </is>
-      </c>
-      <c r="E36" s="4" t="inlineStr">
-        <is>
-          <t>Ingenting — tallene er jo de samme</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>Diagrammet bliver ulovligt</t>
         </is>
       </c>
       <c r="G36" s="4" t="n">
@@ -1537,29 +1537,29 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
+          <t>8 gange</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>2 gange</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>16 gange</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
           <t>4 gange</t>
         </is>
       </c>
-      <c r="D37" s="4" t="inlineStr">
-        <is>
-          <t>2 gange</t>
-        </is>
-      </c>
-      <c r="E37" s="4" t="inlineStr">
-        <is>
-          <t>8 gange</t>
-        </is>
-      </c>
-      <c r="F37" s="4" t="inlineStr">
-        <is>
-          <t>16 gange</t>
-        </is>
-      </c>
       <c r="G37" s="4" t="n">
         <v>30</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="38">
@@ -1573,29 +1573,29 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
+          <t>Gennemsnittet, 98.800 kr</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>Summen af de fem</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>Den højeste løn</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
           <t>Medianen, 24.000 kr</t>
         </is>
       </c>
-      <c r="D38" s="4" t="inlineStr">
-        <is>
-          <t>Gennemsnittet, 98.800 kr</t>
-        </is>
-      </c>
-      <c r="E38" s="4" t="inlineStr">
-        <is>
-          <t>Den højeste løn</t>
-        </is>
-      </c>
-      <c r="F38" s="4" t="inlineStr">
-        <is>
-          <t>Summen af de fem</t>
-        </is>
-      </c>
       <c r="G38" s="4" t="n">
         <v>30</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>